<commit_message>
Rehire Slovakia Code Pk17
</commit_message>
<xml_diff>
--- a/Data/27/TestDataPoland-Regression.xlsx
+++ b/Data/27/TestDataPoland-Regression.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20AC4E65-DF39-4EDC-B724-2533AE486675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D88DBF-ECF8-49DE-8546-1A6E0247D82C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="138">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -273,16 +273,22 @@
     <t>Test_1</t>
   </si>
   <si>
+    <t>10699770</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
     <t>765 Recruitment  (Fihyp Kohawu (10580286))</t>
   </si>
   <si>
     <t>Poland</t>
   </si>
   <si>
-    <t>Stephania</t>
-  </si>
-  <si>
-    <t>Stoltenberg</t>
+    <t>Bo</t>
+  </si>
+  <si>
+    <t>Towne</t>
   </si>
   <si>
     <t xml:space="preserve">698 980 460 </t>
@@ -381,6 +387,9 @@
     <t>ID Card</t>
   </si>
   <si>
+    <t>SSK456211</t>
+  </si>
+  <si>
     <t>Male</t>
   </si>
   <si>
@@ -423,13 +432,13 @@
     <t>765 Store Management (Kires Pivyba (10226524))</t>
   </si>
   <si>
-    <t>Jaylan</t>
-  </si>
-  <si>
-    <t>Jakubowski</t>
-  </si>
-  <si>
-    <t>Auto 29153412</t>
+    <t>Madie</t>
+  </si>
+  <si>
+    <t>Aufderhar</t>
+  </si>
+  <si>
+    <t>Auto 30093495</t>
   </si>
   <si>
     <t>Store Manager_NEW</t>
@@ -447,10 +456,7 @@
     <t xml:space="preserve">251 Management Retail </t>
   </si>
   <si>
-    <t>SSK456202</t>
-  </si>
-  <si>
-    <t>SSK456203</t>
+    <t>SSK456212</t>
   </si>
 </sst>
 </file>
@@ -644,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -779,9 +785,6 @@
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1399,85 +1402,89 @@
       <c r="A2" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="1"/>
+      <c r="B2" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="D2" s="32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E2" s="33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F2" s="34" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G2" s="35" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H2" s="36" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I2" s="36" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J2" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K2" s="37">
         <v>45705</v>
       </c>
       <c r="L2" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="M2" s="36" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="N2" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="O2" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="P2" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q2" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="R2" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="S2" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="T2" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="O2" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="P2" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q2" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="R2" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="S2" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="T2" s="36" t="s">
-        <v>82</v>
-      </c>
       <c r="U2" s="36" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="V2" s="36" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="W2" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="X2" s="38">
         <v>45705</v>
       </c>
       <c r="Y2" s="36" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="Z2" s="36" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AA2" s="36" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AB2" s="36" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AC2" s="36" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AD2" s="36">
         <v>765</v>
@@ -1489,10 +1496,10 @@
         <v>10</v>
       </c>
       <c r="AG2" s="36" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH2" s="36" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AI2" s="18">
         <v>43831</v>
@@ -1501,25 +1508,25 @@
         <v>45293</v>
       </c>
       <c r="AK2" s="36" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AL2" s="36" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AM2" s="36" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AN2" s="40">
         <v>110</v>
       </c>
       <c r="AO2" s="36" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AP2" s="36" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AQ2" s="36" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AR2" s="41">
         <v>45705</v>
@@ -1528,100 +1535,100 @@
         <v>46012</v>
       </c>
       <c r="AT2" s="36" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AU2" s="36" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AV2" s="33" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AW2" s="36" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AX2" s="36" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AY2" s="36" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AZ2" s="36" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BA2" s="36" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BB2" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="BC2" s="36" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="BD2" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BE2" s="33" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BF2" s="15">
-        <v>9577796805</v>
+        <v>9577796902</v>
       </c>
       <c r="BG2" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BH2" s="33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BI2" s="15">
-        <v>49778965435</v>
+        <v>49778965452</v>
       </c>
       <c r="BJ2" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BK2" s="36" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BL2" s="8" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="BM2" s="36" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="BN2" s="42">
         <v>35591</v>
       </c>
       <c r="BO2" s="36" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="BP2" s="36" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="BQ2" s="36" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="BR2" s="36" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="BS2" s="43" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="BT2" s="33" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="BU2" s="44" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="BV2" s="44" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="BW2" s="33" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="BX2" s="33" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="BY2" s="33" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="BZ2" s="5">
         <v>40</v>
@@ -1629,104 +1636,108 @@
     </row>
     <row r="3" spans="1:78" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="1"/>
+        <v>127</v>
+      </c>
+      <c r="B3" s="31">
+        <v>10699771</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="D3" s="32" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F3" s="34" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H3" s="36" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I3" s="40" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J3" s="40" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K3" s="37">
         <f t="shared" ref="K3" ca="1" si="0">TODAY()-31</f>
-        <v>45786</v>
+        <v>45796</v>
       </c>
       <c r="L3" s="33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="M3" s="33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="N3" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="O3" s="45" t="s">
+        <v>87</v>
+      </c>
+      <c r="P3" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q3" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="R3" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="S3" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="T3" s="40" t="s">
         <v>84</v>
       </c>
-      <c r="O3" s="46" t="s">
-        <v>85</v>
-      </c>
-      <c r="P3" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q3" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="R3" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="S3" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="T3" s="40" t="s">
-        <v>82</v>
-      </c>
-      <c r="U3" s="47" t="s">
-        <v>88</v>
-      </c>
-      <c r="V3" s="48" t="s">
-        <v>89</v>
+      <c r="U3" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="V3" s="47" t="s">
+        <v>91</v>
       </c>
       <c r="W3" s="40" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="X3" s="38">
         <f t="shared" ref="X3" ca="1" si="1">K3</f>
-        <v>45786</v>
+        <v>45796</v>
       </c>
       <c r="Y3" s="36" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="Z3" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="AA3" s="49" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB3" s="50" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC3" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="AD3" s="51">
+        <v>131</v>
+      </c>
+      <c r="AA3" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB3" s="49" t="s">
+        <v>132</v>
+      </c>
+      <c r="AC3" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="AD3" s="50">
         <v>765</v>
       </c>
-      <c r="AE3" s="51" t="s">
+      <c r="AE3" s="50" t="s">
         <v>71</v>
       </c>
       <c r="AF3" s="16">
         <v>40</v>
       </c>
       <c r="AG3" s="36" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH3" s="36" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AI3" s="18">
         <v>43831</v>
@@ -1735,25 +1746,25 @@
         <v>45293</v>
       </c>
       <c r="AK3" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="AL3" s="49" t="s">
-        <v>97</v>
+        <v>134</v>
+      </c>
+      <c r="AL3" s="48" t="s">
+        <v>99</v>
       </c>
       <c r="AM3" s="18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AN3" s="40">
         <v>110</v>
       </c>
       <c r="AO3" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="AP3" s="52" t="s">
-        <v>100</v>
+        <v>101</v>
+      </c>
+      <c r="AP3" s="51" t="s">
+        <v>102</v>
       </c>
       <c r="AQ3" s="40" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AR3" s="41">
         <v>45705</v>
@@ -1766,97 +1777,97 @@
         <v>110</v>
       </c>
       <c r="AU3" s="6" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AV3" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AW3" s="36" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AX3" s="36" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AY3" s="36" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AZ3" s="36" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BA3" s="36" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BB3" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="BC3" s="36" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="BD3" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BE3" s="33" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BF3" s="15">
-        <v>9577796806</v>
+        <v>9577796903</v>
       </c>
       <c r="BG3" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BH3" s="33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BI3" s="15">
-        <v>49778965436</v>
+        <v>49778965453</v>
       </c>
       <c r="BJ3" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BK3" s="36" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BL3" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="BM3" s="36" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="BN3" s="42">
         <v>35591</v>
       </c>
       <c r="BO3" s="36" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="BP3" s="36" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="BQ3" s="36" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="BR3" s="36" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="BS3" s="43" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="BT3" s="33" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="BU3" s="44" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="BV3" s="44" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="BW3" s="33" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="BX3" s="33" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="BY3" s="33" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="BZ3" s="5">
         <v>40</v>

</xml_diff>